<commit_message>
Add full dynamic Color / Finish support across Excel mapping, table, modals, and sticker rendering
</commit_message>
<xml_diff>
--- a/rn_valves_template.xlsx
+++ b/rn_valves_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="RN_Box_Stickers" sheetId="1" r:id="rId1"/>
+    <sheet name="RN_Valves_Stickers" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,7 +419,7 @@
         <v>Product Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Collection</v>
+        <v>Color / Finish</v>
       </c>
       <c r="D1" t="str">
         <v>Size</v>
@@ -416,10 +428,10 @@
         <v>MRP</v>
       </c>
       <c r="F1" t="str">
-        <v>Finish</v>
+        <v>Quantity</v>
       </c>
       <c r="G1" t="str">
-        <v>Quantity</v>
+        <v>Collection</v>
       </c>
       <c r="H1" t="str">
         <v>Batch No</v>
@@ -439,7 +451,7 @@
         <v>Angle Cock with Flange</v>
       </c>
       <c r="C2" t="str">
-        <v>G20 Collection</v>
+        <v>Marble</v>
       </c>
       <c r="D2" t="str">
         <v>15mm(1/2")</v>
@@ -447,11 +459,11 @@
       <c r="E2">
         <v>572</v>
       </c>
-      <c r="F2" t="str">
-        <v>Marble</v>
-      </c>
-      <c r="G2">
+      <c r="F2">
         <v>1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>G20 Collection</v>
       </c>
       <c r="H2" t="str">
         <v>RPK06[AASK](02)</v>
@@ -471,19 +483,19 @@
         <v>Bib Cock Heavy with Wall Flange</v>
       </c>
       <c r="C3" t="str">
-        <v>G20 Collection</v>
+        <v>Rose Gold</v>
       </c>
       <c r="D3" t="str">
         <v>15mm (1/2")</v>
       </c>
       <c r="E3">
-        <v>645</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Marble</v>
-      </c>
-      <c r="G3">
+        <v>795</v>
+      </c>
+      <c r="F3">
         <v>2</v>
+      </c>
+      <c r="G3" t="str">
+        <v>G20 Collection</v>
       </c>
       <c r="H3" t="str">
         <v>RPK06[BBSK](01)</v>
@@ -503,7 +515,7 @@
         <v>Brass Ball Valve Heavy Duty</v>
       </c>
       <c r="C4" t="str">
-        <v>Elite Brass Collection</v>
+        <v>Matte Black</v>
       </c>
       <c r="D4" t="str">
         <v>20mm (3/4")</v>
@@ -511,11 +523,11 @@
       <c r="E4">
         <v>1150</v>
       </c>
-      <c r="F4" t="str">
-        <v>Brass Natural</v>
-      </c>
-      <c r="G4">
+      <c r="F4">
         <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Elite Brass Collection</v>
       </c>
       <c r="H4" t="str">
         <v>RPK07[BVHD](05)</v>
@@ -535,7 +547,7 @@
         <v>Concealed Stop Cock (Heavy)</v>
       </c>
       <c r="C5" t="str">
-        <v>G20 Collection</v>
+        <v>Chrome Plated (CP)</v>
       </c>
       <c r="D5" t="str">
         <v>20mm</v>
@@ -543,11 +555,11 @@
       <c r="E5">
         <v>890</v>
       </c>
-      <c r="F5" t="str">
-        <v>Chrome Plated</v>
-      </c>
-      <c r="G5">
+      <c r="F5">
         <v>3</v>
+      </c>
+      <c r="G5" t="str">
+        <v>G20 Collection</v>
       </c>
       <c r="H5" t="str">
         <v>RPK08[CSCK](03)</v>
@@ -567,19 +579,19 @@
         <v>Pillar Cock High Neck</v>
       </c>
       <c r="C6" t="str">
-        <v>G20 Collection</v>
+        <v>Antique Brass</v>
       </c>
       <c r="D6" t="str">
         <v>15mm(1/2")</v>
       </c>
       <c r="E6">
-        <v>1280</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Marble</v>
-      </c>
-      <c r="G6">
+        <v>1480</v>
+      </c>
+      <c r="F6">
         <v>2</v>
+      </c>
+      <c r="G6" t="str">
+        <v>G20 Collection</v>
       </c>
       <c r="H6" t="str">
         <v>RPK09[PCLK](02)</v>
@@ -589,11 +601,43 @@
       </c>
       <c r="J6" t="str">
         <v>3210e76adb2c8899</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>RNSV1015B01</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sink Cock with Swivel Spout</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Gold Finish</v>
+      </c>
+      <c r="D7" t="str">
+        <v>15mm (1/2")</v>
+      </c>
+      <c r="E7">
+        <v>1650</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="str">
+        <v>G20 Collection</v>
+      </c>
+      <c r="H7" t="str">
+        <v>RPK10[SCGV](01)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Jun 2026</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1829f54bca1e7733</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RN Valves Box Sticker v2.0 - Dynamic Pack of and Separate Product Quantity from Print Copies
</commit_message>
<xml_diff>
--- a/rn_valves_template.xlsx
+++ b/rn_valves_template.xlsx
@@ -397,18 +397,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,24 +423,27 @@
         <v>Color / Finish</v>
       </c>
       <c r="D1" t="str">
+        <v>Product Qty (On Sticker)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Print Copies (Stickers Count)</v>
+      </c>
+      <c r="F1" t="str">
         <v>Size</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>MRP</v>
       </c>
-      <c r="F1" t="str">
-        <v>Quantity</v>
-      </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Collection</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Batch No</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>MFG Date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>sku-code</v>
       </c>
     </row>
@@ -454,24 +458,27 @@
         <v>Marble</v>
       </c>
       <c r="D2" t="str">
+        <v>1 N</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2" t="str">
         <v>15mm(1/2")</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>572</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>G20 Collection</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>RPK06[AASK](02)</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>7646a28acb8c3349</v>
       </c>
     </row>
@@ -486,24 +493,27 @@
         <v>Rose Gold</v>
       </c>
       <c r="D3" t="str">
+        <v>Pack of 2</v>
+      </c>
+      <c r="E3">
+        <v>50</v>
+      </c>
+      <c r="F3" t="str">
         <v>15mm (1/2")</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>795</v>
       </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>G20 Collection</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>RPK06[BBSK](01)</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>8752b39bdf9d4451</v>
       </c>
     </row>
@@ -518,24 +528,27 @@
         <v>Matte Black</v>
       </c>
       <c r="D4" t="str">
+        <v>Pack of 3</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="F4" t="str">
         <v>20mm (3/4")</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>1150</v>
       </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Elite Brass Collection</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>RPK07[BVHD](05)</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>9120c48cfe1e5562</v>
       </c>
     </row>
@@ -550,24 +563,27 @@
         <v>Chrome Plated (CP)</v>
       </c>
       <c r="D5" t="str">
+        <v>Pack of 2</v>
+      </c>
+      <c r="E5">
+        <v>30</v>
+      </c>
+      <c r="F5" t="str">
         <v>20mm</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>890</v>
       </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>G20 Collection</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>RPK08[CSCK](03)</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>6543d21bca9a1122</v>
       </c>
     </row>
@@ -582,24 +598,27 @@
         <v>Antique Brass</v>
       </c>
       <c r="D6" t="str">
+        <v>1 N</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6" t="str">
         <v>15mm(1/2")</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>1480</v>
       </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>G20 Collection</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>RPK09[PCLK](02)</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>3210e76adb2c8899</v>
       </c>
     </row>
@@ -614,30 +633,33 @@
         <v>Gold Finish</v>
       </c>
       <c r="D7" t="str">
+        <v>Pack of 4</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+      <c r="F7" t="str">
         <v>15mm (1/2")</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>1650</v>
       </c>
-      <c r="F7">
-        <v>2</v>
-      </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>G20 Collection</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>RPK10[SCGV](01)</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>Jun 2026</v>
       </c>
-      <c r="J7" t="str">
+      <c r="K7" t="str">
         <v>1829f54bca1e7733</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>